<commit_message>
updated events normalized xlsx
</commit_message>
<xml_diff>
--- a/week-02/Ex2A_events_normalized.xlsx
+++ b/week-02/Ex2A_events_normalized.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chimm\Documents\DataAnalytics-2026\week-02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4DA49493-854C-4FFA-B609-4A6EF920F4BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3029436A-DF0B-402E-9851-9949898F9806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5091876E-AF08-41C4-B976-D2AB9D8B455C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5091876E-AF08-41C4-B976-D2AB9D8B455C}"/>
   </bookViews>
   <sheets>
     <sheet name="events_sample" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="131">
   <si>
     <t>Event ID</t>
   </si>
@@ -416,13 +416,16 @@
     <t>Event Table</t>
   </si>
   <si>
-    <t>Locatoin Table</t>
-  </si>
-  <si>
     <t>Venue Table</t>
   </si>
   <si>
     <t>Employee Table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category Table </t>
+  </si>
+  <si>
+    <t>Elenda Rodriguez</t>
   </si>
 </sst>
 </file>
@@ -927,13 +930,14 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1314,11 +1318,12 @@
   <cols>
     <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.109375" customWidth="1"/>
+    <col min="4" max="4" width="29.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.109375" customWidth="1"/>
+    <col min="6" max="6" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.21875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="32.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.44140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15.5546875" bestFit="1" customWidth="1"/>
@@ -1973,739 +1978,736 @@
         <v>100</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" s="5" t="s">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="C17" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B18" s="5">
         <v>1</v>
       </c>
-      <c r="D17" t="s">
-        <v>103</v>
-      </c>
-      <c r="E17" t="s">
+      <c r="C18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B19" s="5">
         <v>2</v>
       </c>
-      <c r="F17" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="5">
-        <v>102</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="C19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B20" s="5">
         <v>3</v>
       </c>
-      <c r="D18" t="s">
+      <c r="C20" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B21" s="5">
+        <v>4</v>
+      </c>
+      <c r="C21" t="s">
+        <v>22</v>
+      </c>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B22" s="5">
         <v>5</v>
       </c>
-      <c r="E18" s="1">
-        <v>46095</v>
-      </c>
-      <c r="F18" t="s">
+      <c r="C22" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B23" s="5">
         <v>6</v>
       </c>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="5">
-        <v>103</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="C23" t="s">
+        <v>19</v>
+      </c>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B24" s="5">
         <v>7</v>
       </c>
-      <c r="D19" t="s">
+      <c r="C24" t="s">
         <v>5</v>
       </c>
-      <c r="E19" s="1">
-        <v>46194</v>
-      </c>
-      <c r="F19" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="5">
-        <v>104</v>
-      </c>
-      <c r="C20" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" t="s">
-        <v>12</v>
-      </c>
-      <c r="E20" s="1">
-        <v>46115</v>
-      </c>
-      <c r="F20" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="5">
-        <v>105</v>
-      </c>
-      <c r="C21" t="s">
-        <v>14</v>
-      </c>
-      <c r="D21" t="s">
-        <v>16</v>
-      </c>
-      <c r="E21" s="1">
-        <v>46157</v>
-      </c>
-      <c r="F21" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="5">
-        <v>106</v>
-      </c>
-      <c r="C22" t="s">
-        <v>17</v>
-      </c>
-      <c r="D22" t="s">
-        <v>19</v>
-      </c>
-      <c r="E22" s="1">
-        <v>46109</v>
-      </c>
-      <c r="F22" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="5">
-        <v>107</v>
-      </c>
-      <c r="C23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E23" s="1">
-        <v>46130</v>
-      </c>
-      <c r="F23" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B24" s="5">
-        <v>108</v>
-      </c>
-      <c r="C24" t="s">
-        <v>24</v>
-      </c>
-      <c r="D24" t="s">
-        <v>26</v>
-      </c>
-      <c r="E24" s="1">
-        <v>46144</v>
-      </c>
-      <c r="F24" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B25" s="5">
-        <v>109</v>
-      </c>
-      <c r="C25" t="s">
-        <v>27</v>
-      </c>
-      <c r="D25" t="s">
-        <v>16</v>
-      </c>
-      <c r="E25" s="1">
-        <v>46181</v>
-      </c>
-      <c r="F25" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="5">
-        <v>110</v>
-      </c>
-      <c r="C26" t="s">
-        <v>30</v>
-      </c>
-      <c r="D26" t="s">
-        <v>5</v>
-      </c>
-      <c r="E26" s="1">
-        <v>46215</v>
-      </c>
-      <c r="F26" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B27" s="5">
-        <v>111</v>
-      </c>
-      <c r="C27" t="s">
-        <v>31</v>
-      </c>
-      <c r="D27" t="s">
-        <v>12</v>
-      </c>
-      <c r="E27" s="1">
-        <v>46102</v>
-      </c>
-      <c r="F27" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B28" s="5">
-        <v>112</v>
-      </c>
-      <c r="C28" t="s">
-        <v>33</v>
-      </c>
-      <c r="D28" t="s">
-        <v>35</v>
-      </c>
-      <c r="E28" s="1">
-        <v>46137</v>
-      </c>
-      <c r="F28" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E25" s="1"/>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E26" s="1"/>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E27" s="1"/>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E28" s="1"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>101</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B34" s="5" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C34" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D34" t="s">
-        <v>90</v>
-      </c>
-      <c r="E34" t="s">
-        <v>91</v>
-      </c>
-      <c r="F34" t="s">
-        <v>92</v>
-      </c>
-      <c r="G34" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B35" s="5">
-        <v>7</v>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B35" s="5" t="s">
+        <v>108</v>
       </c>
       <c r="C35" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D35" t="s">
-        <v>42</v>
-      </c>
-      <c r="E35" t="s">
-        <v>43</v>
-      </c>
-      <c r="F35" t="s">
-        <v>44</v>
-      </c>
-      <c r="G35">
-        <v>90026</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B36" s="5">
-        <v>7</v>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B36" s="5" t="s">
+        <v>109</v>
       </c>
       <c r="C36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D36" t="s">
-        <v>47</v>
-      </c>
-      <c r="E36" t="s">
-        <v>48</v>
-      </c>
-      <c r="F36" t="s">
-        <v>49</v>
-      </c>
-      <c r="G36">
-        <v>78741</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B37" s="5">
-        <v>2</v>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B37" s="5" t="s">
+        <v>110</v>
       </c>
       <c r="C37" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D37" t="s">
-        <v>53</v>
-      </c>
-      <c r="E37" t="s">
-        <v>54</v>
-      </c>
-      <c r="F37" t="s">
-        <v>44</v>
-      </c>
-      <c r="G37">
-        <v>90046</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B38" s="5">
-        <v>3</v>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B38" s="5" t="s">
+        <v>125</v>
       </c>
       <c r="C38" t="s">
-        <v>15</v>
+        <v>130</v>
       </c>
       <c r="D38" t="s">
-        <v>57</v>
-      </c>
-      <c r="E38" t="s">
-        <v>58</v>
-      </c>
-      <c r="F38" t="s">
-        <v>59</v>
-      </c>
-      <c r="G38">
-        <v>60616</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B39" s="5">
-        <v>6</v>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B39" s="5" t="s">
+        <v>111</v>
       </c>
       <c r="C39" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D39" t="s">
-        <v>63</v>
-      </c>
-      <c r="E39" t="s">
-        <v>64</v>
-      </c>
-      <c r="F39" t="s">
-        <v>65</v>
-      </c>
-      <c r="G39">
-        <v>10011</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B40" s="5">
-        <v>4</v>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B40" s="5" t="s">
+        <v>112</v>
       </c>
       <c r="C40" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="D40" t="s">
-        <v>57</v>
-      </c>
-      <c r="E40" t="s">
-        <v>58</v>
-      </c>
-      <c r="F40" t="s">
-        <v>59</v>
-      </c>
-      <c r="G40">
-        <v>60616</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B41" s="5">
-        <v>5</v>
-      </c>
-      <c r="C41" t="s">
-        <v>25</v>
-      </c>
-      <c r="D41" t="s">
-        <v>69</v>
-      </c>
-      <c r="E41" t="s">
-        <v>70</v>
-      </c>
-      <c r="F41" t="s">
-        <v>71</v>
-      </c>
-      <c r="G41">
-        <v>97214</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B42" s="5">
-        <v>3</v>
-      </c>
-      <c r="C42" t="s">
-        <v>28</v>
-      </c>
-      <c r="D42" t="s">
-        <v>75</v>
-      </c>
-      <c r="E42" t="s">
-        <v>76</v>
-      </c>
-      <c r="F42" t="s">
-        <v>77</v>
-      </c>
-      <c r="G42">
-        <v>48226</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B43" s="5">
-        <v>7</v>
-      </c>
-      <c r="C43" t="s">
-        <v>4</v>
-      </c>
-      <c r="D43" t="s">
-        <v>42</v>
-      </c>
-      <c r="E43" t="s">
-        <v>43</v>
-      </c>
-      <c r="F43" t="s">
-        <v>44</v>
-      </c>
-      <c r="G43">
-        <v>90026</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B44" s="5">
-        <v>2</v>
-      </c>
-      <c r="C44" t="s">
-        <v>32</v>
-      </c>
-      <c r="D44" t="s">
-        <v>81</v>
-      </c>
-      <c r="E44" t="s">
-        <v>64</v>
-      </c>
-      <c r="F44" t="s">
-        <v>65</v>
-      </c>
-      <c r="G44">
-        <v>10012</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B45" s="5">
-        <v>1</v>
-      </c>
-      <c r="C45" t="s">
-        <v>34</v>
-      </c>
-      <c r="D45" t="s">
-        <v>84</v>
-      </c>
-      <c r="E45" t="s">
-        <v>85</v>
-      </c>
-      <c r="F45" t="s">
-        <v>86</v>
-      </c>
-      <c r="G45">
-        <v>33132</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B41" s="6"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B42" s="6"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B43" s="6"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B44" s="6"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B45" s="6"/>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
         <v>102</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B51" s="5" t="s">
         <v>114</v>
       </c>
       <c r="C51" t="s">
+        <v>113</v>
+      </c>
+      <c r="D51" t="s">
+        <v>90</v>
+      </c>
+      <c r="E51" t="s">
+        <v>91</v>
+      </c>
+      <c r="F51" t="s">
+        <v>92</v>
+      </c>
+      <c r="G51" t="s">
+        <v>93</v>
+      </c>
+      <c r="H51" t="s">
         <v>96</v>
       </c>
-      <c r="D51" t="s">
+      <c r="I51" t="s">
         <v>94</v>
       </c>
-      <c r="E51" t="s">
+      <c r="J51" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B52" s="5" t="s">
         <v>116</v>
       </c>
       <c r="C52" t="s">
+        <v>4</v>
+      </c>
+      <c r="D52" t="s">
+        <v>42</v>
+      </c>
+      <c r="E52" t="s">
+        <v>43</v>
+      </c>
+      <c r="F52" t="s">
+        <v>44</v>
+      </c>
+      <c r="G52">
+        <v>90026</v>
+      </c>
+      <c r="H52" t="s">
         <v>98</v>
       </c>
-      <c r="D52" t="s">
+      <c r="I52" t="s">
         <v>45</v>
       </c>
-      <c r="E52" t="s">
+      <c r="J52" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B53" s="5" t="s">
         <v>115</v>
       </c>
       <c r="C53" t="s">
+        <v>8</v>
+      </c>
+      <c r="D53" t="s">
+        <v>47</v>
+      </c>
+      <c r="E53" t="s">
+        <v>48</v>
+      </c>
+      <c r="F53" t="s">
+        <v>49</v>
+      </c>
+      <c r="G53">
+        <v>78741</v>
+      </c>
+      <c r="H53" t="s">
         <v>50</v>
       </c>
-      <c r="D53" t="s">
+      <c r="I53" t="s">
         <v>51</v>
       </c>
-      <c r="E53" t="s">
+      <c r="J53" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B54" s="5" t="s">
         <v>117</v>
       </c>
       <c r="C54" t="s">
+        <v>11</v>
+      </c>
+      <c r="D54" t="s">
+        <v>53</v>
+      </c>
+      <c r="E54" t="s">
+        <v>54</v>
+      </c>
+      <c r="F54" t="s">
+        <v>44</v>
+      </c>
+      <c r="G54">
+        <v>90046</v>
+      </c>
+      <c r="H54" t="s">
         <v>99</v>
       </c>
-      <c r="D54" t="s">
+      <c r="I54" t="s">
         <v>55</v>
       </c>
-      <c r="E54" t="s">
+      <c r="J54" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B55" s="5" t="s">
         <v>118</v>
       </c>
       <c r="C55" t="s">
+        <v>15</v>
+      </c>
+      <c r="D55" t="s">
+        <v>57</v>
+      </c>
+      <c r="E55" t="s">
+        <v>58</v>
+      </c>
+      <c r="F55" t="s">
+        <v>59</v>
+      </c>
+      <c r="G55">
+        <v>60616</v>
+      </c>
+      <c r="H55" t="s">
         <v>60</v>
       </c>
-      <c r="D55" t="s">
+      <c r="I55" t="s">
         <v>61</v>
       </c>
-      <c r="E55" t="s">
+      <c r="J55" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B56" s="5" t="s">
         <v>119</v>
       </c>
       <c r="C56" t="s">
+        <v>18</v>
+      </c>
+      <c r="D56" t="s">
+        <v>63</v>
+      </c>
+      <c r="E56" t="s">
+        <v>64</v>
+      </c>
+      <c r="F56" t="s">
+        <v>65</v>
+      </c>
+      <c r="G56">
+        <v>10011</v>
+      </c>
+      <c r="H56" t="s">
         <v>66</v>
       </c>
-      <c r="D56" t="s">
+      <c r="I56" t="s">
         <v>67</v>
       </c>
-      <c r="E56" t="s">
+      <c r="J56" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B57" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C57" t="s">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="D57" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E57" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+      <c r="F57" t="s">
+        <v>71</v>
+      </c>
+      <c r="G57">
+        <v>97214</v>
+      </c>
+      <c r="H57" t="s">
+        <v>72</v>
+      </c>
+      <c r="I57" t="s">
+        <v>73</v>
+      </c>
+      <c r="J57" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B58" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C58" t="s">
-        <v>72</v>
+        <v>28</v>
       </c>
       <c r="D58" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E58" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+      <c r="F58" t="s">
+        <v>77</v>
+      </c>
+      <c r="G58">
+        <v>48226</v>
+      </c>
+      <c r="H58" t="s">
+        <v>78</v>
+      </c>
+      <c r="I58" t="s">
+        <v>79</v>
+      </c>
+      <c r="J58" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B59" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C59" t="s">
-        <v>78</v>
+        <v>32</v>
       </c>
       <c r="D59" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E59" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="F59" t="s">
+        <v>65</v>
+      </c>
+      <c r="G59">
+        <v>10012</v>
+      </c>
+      <c r="H59" t="s">
+        <v>97</v>
+      </c>
+      <c r="I59" t="s">
+        <v>82</v>
+      </c>
+      <c r="J59" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B60" s="5" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C60" t="s">
-        <v>98</v>
+        <v>34</v>
       </c>
       <c r="D60" t="s">
-        <v>45</v>
+        <v>84</v>
       </c>
       <c r="E60" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B61" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="C61" t="s">
-        <v>97</v>
-      </c>
-      <c r="D61" t="s">
-        <v>82</v>
-      </c>
-      <c r="E61" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B62" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="C62" t="s">
+        <v>85</v>
+      </c>
+      <c r="F60" t="s">
+        <v>86</v>
+      </c>
+      <c r="G60">
+        <v>33132</v>
+      </c>
+      <c r="H60" t="s">
         <v>87</v>
       </c>
-      <c r="D62" t="s">
+      <c r="I60" t="s">
         <v>88</v>
       </c>
-      <c r="E62" t="s">
+      <c r="J60" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
         <v>124</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B68" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C68" t="s">
+        <v>1</v>
+      </c>
+      <c r="D68" t="s">
+        <v>2</v>
+      </c>
+      <c r="E68" t="s">
+        <v>104</v>
+      </c>
+      <c r="F68" t="s">
         <v>107</v>
       </c>
-      <c r="C68" t="s">
+      <c r="G68" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B69" s="5">
+        <v>102</v>
+      </c>
+      <c r="C69" t="s">
+        <v>3</v>
+      </c>
+      <c r="D69" s="1">
+        <v>46095</v>
+      </c>
+      <c r="E69">
+        <v>7</v>
+      </c>
+      <c r="F69" t="s">
+        <v>108</v>
+      </c>
+      <c r="G69" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B70" s="5">
+        <v>103</v>
+      </c>
+      <c r="C70" t="s">
+        <v>7</v>
+      </c>
+      <c r="D70" s="1">
+        <v>46194</v>
+      </c>
+      <c r="E70">
+        <v>7</v>
+      </c>
+      <c r="F70" t="s">
+        <v>109</v>
+      </c>
+      <c r="G70" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B71" s="5">
+        <v>104</v>
+      </c>
+      <c r="C71" t="s">
+        <v>10</v>
+      </c>
+      <c r="D71" s="1">
+        <v>46115</v>
+      </c>
+      <c r="E71">
+        <v>2</v>
+      </c>
+      <c r="F71" t="s">
+        <v>110</v>
+      </c>
+      <c r="G71" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B72" s="5">
+        <v>105</v>
+      </c>
+      <c r="C72" t="s">
+        <v>14</v>
+      </c>
+      <c r="D72" s="1">
+        <v>46157</v>
+      </c>
+      <c r="E72">
+        <v>3</v>
+      </c>
+      <c r="F72" t="s">
+        <v>109</v>
+      </c>
+      <c r="G72" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B73" s="5">
         <v>106</v>
       </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B69" s="5" t="s">
+      <c r="C73" t="s">
+        <v>17</v>
+      </c>
+      <c r="D73" s="1">
+        <v>46109</v>
+      </c>
+      <c r="E73">
+        <v>6</v>
+      </c>
+      <c r="F73" t="s">
+        <v>125</v>
+      </c>
+      <c r="G73" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B74" s="5">
+        <v>107</v>
+      </c>
+      <c r="C74" t="s">
+        <v>21</v>
+      </c>
+      <c r="D74" s="1">
+        <v>46130</v>
+      </c>
+      <c r="E74">
+        <v>4</v>
+      </c>
+      <c r="F74" t="s">
+        <v>111</v>
+      </c>
+      <c r="G74" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B75" s="5">
         <v>108</v>
       </c>
-      <c r="C69" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B70" s="5" t="s">
+      <c r="C75" t="s">
+        <v>24</v>
+      </c>
+      <c r="D75" s="1">
+        <v>46144</v>
+      </c>
+      <c r="E75">
+        <v>5</v>
+      </c>
+      <c r="F75" t="s">
+        <v>110</v>
+      </c>
+      <c r="G75" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B76" s="5">
         <v>109</v>
       </c>
-      <c r="C70" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B71" s="5" t="s">
+      <c r="C76" t="s">
+        <v>27</v>
+      </c>
+      <c r="D76" s="1">
+        <v>46181</v>
+      </c>
+      <c r="E76">
+        <v>3</v>
+      </c>
+      <c r="F76" t="s">
+        <v>112</v>
+      </c>
+      <c r="G76" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B77" s="5">
         <v>110</v>
       </c>
-      <c r="C71" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B72" s="5" t="s">
+      <c r="C77" t="s">
+        <v>30</v>
+      </c>
+      <c r="D77" s="1">
+        <v>46215</v>
+      </c>
+      <c r="E77">
+        <v>7</v>
+      </c>
+      <c r="F77" t="s">
         <v>109</v>
       </c>
-      <c r="C72" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B73" s="5" t="s">
+      <c r="G77" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B78" s="5">
+        <v>111</v>
+      </c>
+      <c r="C78" t="s">
+        <v>31</v>
+      </c>
+      <c r="D78" s="1">
+        <v>46102</v>
+      </c>
+      <c r="E78">
+        <v>2</v>
+      </c>
+      <c r="F78" t="s">
+        <v>110</v>
+      </c>
+      <c r="G78" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B79" s="5">
+        <v>112</v>
+      </c>
+      <c r="C79" t="s">
+        <v>33</v>
+      </c>
+      <c r="D79" s="1">
+        <v>46137</v>
+      </c>
+      <c r="E79">
+        <v>1</v>
+      </c>
+      <c r="F79" t="s">
         <v>125</v>
       </c>
-      <c r="C73" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B74" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C74" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B75" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C75" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B76" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C76" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B77" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="C77" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B78" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C78" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B79" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="C79" t="s">
-        <v>39</v>
+      <c r="G79" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2717,15 +2719,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CA5D0A6329BB324E86983B32928CFC2E" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d7eac4bce3bbb09c82bd908806be82e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9e0b35a9-e6cb-436b-81d4-4440ba439ca5" xmlns:ns3="ced60a7f-99b1-48d2-b555-34851c8026ae" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb51570e5b7cb8bd524bc2df5324d4a3" ns2:_="" ns3:_="">
     <xsd:import namespace="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
@@ -2966,6 +2959,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2978,14 +2980,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D48FB9E6-6DE3-40FB-81F7-677295638F7C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6414E68-BBC1-4A96-B078-EF7EE95D29CE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3004,6 +2998,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D48FB9E6-6DE3-40FB-81F7-677295638F7C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EE6EC55-B0E7-4ACE-A5DA-E03DCA4973DE}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
updating events normalized xlsx
</commit_message>
<xml_diff>
--- a/week-02/Ex2A_events_normalized.xlsx
+++ b/week-02/Ex2A_events_normalized.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chimm\Documents\DataAnalytics-2026\week-02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3029436A-DF0B-402E-9851-9949898F9806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5815B00C-7DD2-4BE6-ABDE-D5897D7BFF7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5091876E-AF08-41C4-B976-D2AB9D8B455C}"/>
   </bookViews>
@@ -930,14 +930,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2149,21 +2148,6 @@
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B41" s="6"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B42" s="6"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B43" s="6"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B44" s="6"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B45" s="6"/>
-    </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
         <v>102</v>
@@ -2719,6 +2703,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CA5D0A6329BB324E86983B32928CFC2E" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d7eac4bce3bbb09c82bd908806be82e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9e0b35a9-e6cb-436b-81d4-4440ba439ca5" xmlns:ns3="ced60a7f-99b1-48d2-b555-34851c8026ae" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb51570e5b7cb8bd524bc2df5324d4a3" ns2:_="" ns3:_="">
     <xsd:import namespace="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
@@ -2959,15 +2952,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2980,6 +2964,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D48FB9E6-6DE3-40FB-81F7-677295638F7C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6414E68-BBC1-4A96-B078-EF7EE95D29CE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2998,14 +2990,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D48FB9E6-6DE3-40FB-81F7-677295638F7C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EE6EC55-B0E7-4ACE-A5DA-E03DCA4973DE}">
   <ds:schemaRefs>

</xml_diff>